<commit_message>
adding the data to the site and adding another mutate case
</commit_message>
<xml_diff>
--- a/docs/content/codebook.xlsx
+++ b/docs/content/codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mariafinnsdottir/Documents/GitHub/r-clusters-may2026/docs/content/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEE6A0AD-A8FB-D34F-AEC6-E7A037F7F04C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2D1857-A384-0F45-8B54-A1FFB6F3393D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36700" yWindow="-1120" windowWidth="26340" windowHeight="18740" xr2:uid="{A8DD527A-C240-3947-9345-FC4C5F293D65}"/>
+    <workbookView xWindow="5580" yWindow="2380" windowWidth="23820" windowHeight="15440" xr2:uid="{A8DD527A-C240-3947-9345-FC4C5F293D65}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="97">
   <si>
     <t>WVS variable label</t>
   </si>
@@ -56,15 +56,6 @@
     <t>Q49</t>
   </si>
   <si>
-    <t>Q50</t>
-  </si>
-  <si>
-    <t>Q56</t>
-  </si>
-  <si>
-    <t>Q178</t>
-  </si>
-  <si>
     <t>Q207</t>
   </si>
   <si>
@@ -107,21 +98,12 @@
     <t>life_satis</t>
   </si>
   <si>
-    <t>finance_satis</t>
-  </si>
-  <si>
-    <t>stand_living</t>
-  </si>
-  <si>
     <t>numeric</t>
   </si>
   <si>
     <t>1 through 10 where 1 is completely dissatisfied and 10 is completely satisfied</t>
   </si>
   <si>
-    <t>avoid_fare</t>
-  </si>
-  <si>
     <t>social_media</t>
   </si>
   <si>
@@ -140,9 +122,6 @@
     <t>education</t>
   </si>
   <si>
-    <t>employed</t>
-  </si>
-  <si>
     <t>sector</t>
   </si>
   <si>
@@ -179,18 +158,6 @@
     <t>Satisfaction with your life</t>
   </si>
   <si>
-    <t>Satisfaction with the financial situation of your household</t>
-  </si>
-  <si>
-    <t>Standard of living compared with your parents</t>
-  </si>
-  <si>
-    <t>1 through 10 where 1 is never justifiable and 10 is always justifiable</t>
-  </si>
-  <si>
-    <t>Justifiable: Avoiding a fare on public transport</t>
-  </si>
-  <si>
     <t>Information source: Social media</t>
   </si>
   <si>
@@ -227,15 +194,6 @@
     <t>Very good</t>
   </si>
   <si>
-    <t>Better off</t>
-  </si>
-  <si>
-    <t>About the same</t>
-  </si>
-  <si>
-    <t>Worse off</t>
-  </si>
-  <si>
     <t>Daily</t>
   </si>
   <si>
@@ -369,6 +327,9 @@
   </si>
   <si>
     <t xml:space="preserve">Upper class </t>
+  </si>
+  <si>
+    <t>emp_status</t>
   </si>
 </sst>
 </file>
@@ -747,7 +708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F715AF9-FE40-2D4E-AE51-43627CC8081D}">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -755,16 +716,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="E1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -772,16 +733,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -789,16 +750,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="H3" s="1"/>
     </row>
@@ -807,40 +768,40 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E5" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E6" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="H6" s="1"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E7" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="H7" s="1"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E8" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="H8" s="1"/>
     </row>
@@ -849,16 +810,16 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H9" s="1"/>
     </row>
@@ -867,106 +828,106 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="H10" s="1"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" t="s">
-        <v>47</v>
-      </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="H11" s="1"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E12" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="H12" s="1"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E13" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="H13" s="1"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" t="s">
-        <v>49</v>
-      </c>
       <c r="E14" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="H14" s="1"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D15" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="H15" s="1"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E16" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="H16" s="1"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" t="s">
+        <v>42</v>
+      </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="H17" s="1"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>43</v>
+      </c>
       <c r="E18" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="H18" s="1"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E19" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="H19" s="1"/>
     </row>
@@ -975,288 +936,222 @@
         <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D20" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E20" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H20" s="1"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E21" t="s">
-        <v>71</v>
-      </c>
-      <c r="H21" s="1"/>
+        <v>61</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22" t="s">
-        <v>24</v>
-      </c>
-      <c r="D22" t="s">
-        <v>53</v>
-      </c>
       <c r="E22" t="s">
-        <v>52</v>
-      </c>
-      <c r="H22" s="1"/>
+        <v>62</v>
+      </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>11</v>
-      </c>
-      <c r="B23" t="s">
-        <v>30</v>
-      </c>
-      <c r="C23" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" t="s">
-        <v>54</v>
-      </c>
       <c r="E23" t="s">
-        <v>72</v>
-      </c>
-      <c r="H23" s="1"/>
+        <v>63</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E24" t="s">
-        <v>73</v>
-      </c>
-      <c r="H24" s="1"/>
+        <v>64</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B25" t="s">
-        <v>31</v>
-      </c>
-      <c r="C25" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" t="s">
-        <v>55</v>
-      </c>
       <c r="E25" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s">
+        <v>66</v>
+      </c>
+      <c r="E26" t="s">
         <v>74</v>
-      </c>
-      <c r="H25" s="1"/>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E26" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E27" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E28" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E29" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E30" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>13</v>
-      </c>
-      <c r="B31" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" t="s">
-        <v>41</v>
-      </c>
-      <c r="D31" t="s">
-        <v>80</v>
-      </c>
       <c r="E31" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E32" t="s">
-        <v>87</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E33" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E34" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E35" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" t="s">
+        <v>96</v>
+      </c>
+      <c r="C36" t="s">
+        <v>76</v>
+      </c>
       <c r="E36" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E37" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E38" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E39" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E40" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>14</v>
-      </c>
-      <c r="B41" t="s">
-        <v>33</v>
-      </c>
-      <c r="C41" t="s">
-        <v>90</v>
-      </c>
       <c r="E41" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E42" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E43" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" t="s">
+        <v>27</v>
+      </c>
+      <c r="C44" t="s">
+        <v>34</v>
+      </c>
+      <c r="D44" t="s">
+        <v>85</v>
+      </c>
       <c r="E44" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E45" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E46" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="E47" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C48" t="s">
+        <v>34</v>
+      </c>
+      <c r="D48" t="s">
+        <v>90</v>
+      </c>
       <c r="E48" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>15</v>
-      </c>
-      <c r="B49" t="s">
-        <v>34</v>
-      </c>
-      <c r="C49" t="s">
-        <v>41</v>
-      </c>
-      <c r="D49" t="s">
-        <v>99</v>
-      </c>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E49" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E50" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E51" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E52" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>16</v>
-      </c>
-      <c r="B53" t="s">
-        <v>35</v>
-      </c>
-      <c r="C53" t="s">
-        <v>41</v>
-      </c>
-      <c r="D53" t="s">
-        <v>104</v>
-      </c>
-      <c r="E53" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="E54" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="E55" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="E56" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="E57" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>